<commit_message>
artist list component and duplicate structure to all years for now
</commit_message>
<xml_diff>
--- a/data/lineup-2025.xlsx
+++ b/data/lineup-2025.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/pekkos/git/bingsjostamman.se/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AFF95324-ECF2-8449-B7BF-2DE4B843F884}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35FB7CEB-45F3-8847-97E0-8D02117BBAE9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="67420" yWindow="10660" windowWidth="36000" windowHeight="21480" xr2:uid="{60F76CC9-F7FE-B34D-9EF7-EFD856BA5ECF}"/>
+    <workbookView xWindow="0" yWindow="680" windowWidth="30240" windowHeight="18960" xr2:uid="{60F76CC9-F7FE-B34D-9EF7-EFD856BA5ECF}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="224" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="230" uniqueCount="95">
   <si>
     <t>day</t>
   </si>
@@ -104,9 +104,6 @@
     <t>Se Bingsjödräkten i olika skepnader.</t>
   </si>
   <si>
-    <t>Tvallmusikinstrument</t>
-  </si>
-  <si>
     <t>Träffa en byggare av vallmusikinstrument</t>
   </si>
   <si>
@@ -122,9 +119,6 @@
     <t>Långdans och balladdans</t>
   </si>
   <si>
-    <t>Bystugebanan</t>
-  </si>
-  <si>
     <t>Prova på polska</t>
   </si>
   <si>
@@ -140,18 +134,6 @@
     <t>Låttältet</t>
   </si>
   <si>
-    <t>Bingsjölåtar med Täby spelmansgille</t>
-  </si>
-  <si>
-    <t>Orelåtar med Ore spelmän</t>
-  </si>
-  <si>
-    <t>Norra Hälsingland med Nordanstigs spelmanslag</t>
-  </si>
-  <si>
-    <t>Rättvikslåtar med Rättviks spelmanslag</t>
-  </si>
-  <si>
     <t>Södra Dalarna med Korsmora spelmän</t>
   </si>
   <si>
@@ -315,6 +297,30 @@
   </si>
   <si>
     <t>artist</t>
+  </si>
+  <si>
+    <t>Vallmusikinstrument</t>
+  </si>
+  <si>
+    <t>Bingsjölåtar</t>
+  </si>
+  <si>
+    <t>Ore spelmän</t>
+  </si>
+  <si>
+    <t>Orelåtar</t>
+  </si>
+  <si>
+    <t>Låtar från södra Dalarna</t>
+  </si>
+  <si>
+    <t>Låtar från Norra Hälsingland</t>
+  </si>
+  <si>
+    <t>Rättvis spelmanslag</t>
+  </si>
+  <si>
+    <t>Rättvikslåtar</t>
   </si>
 </sst>
 </file>
@@ -734,19 +740,19 @@
         <v>6</v>
       </c>
       <c r="E1" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="F1" t="s">
+        <v>77</v>
+      </c>
+      <c r="G1" t="s">
         <v>83</v>
-      </c>
-      <c r="G1" t="s">
-        <v>89</v>
       </c>
       <c r="H1" t="s">
         <v>1</v>
       </c>
       <c r="I1" t="s">
-        <v>90</v>
+        <v>84</v>
       </c>
       <c r="J1" s="3" t="s">
         <v>2</v>
@@ -755,7 +761,7 @@
         <v>9</v>
       </c>
       <c r="L1" s="3" t="s">
-        <v>82</v>
+        <v>76</v>
       </c>
       <c r="M1" t="s">
         <v>3</v>
@@ -775,22 +781,25 @@
         <v>10</v>
       </c>
       <c r="E2" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="G2" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="H2" t="s">
         <v>11</v>
       </c>
       <c r="I2" t="s">
-        <v>91</v>
+        <v>85</v>
       </c>
       <c r="J2" s="3" t="s">
         <v>12</v>
       </c>
       <c r="K2" s="1" t="s">
         <v>13</v>
+      </c>
+      <c r="M2" s="4" t="s">
+        <v>80</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.2">
@@ -807,10 +816,10 @@
         <v>10</v>
       </c>
       <c r="E3" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="G3" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="H3" t="s">
         <v>16</v>
@@ -831,10 +840,10 @@
         <v>10</v>
       </c>
       <c r="E4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="G4" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="H4" t="s">
         <v>17</v>
@@ -858,7 +867,7 @@
         <v>19</v>
       </c>
       <c r="E5" t="s">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="H5" t="s">
         <v>20</v>
@@ -882,13 +891,13 @@
         <v>19</v>
       </c>
       <c r="E6" t="s">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="H6" t="s">
+        <v>87</v>
+      </c>
+      <c r="J6" s="3" t="s">
         <v>22</v>
-      </c>
-      <c r="J6" s="3" t="s">
-        <v>23</v>
       </c>
       <c r="K6" s="1"/>
     </row>
@@ -903,16 +912,16 @@
         <v>0.70833333333333337</v>
       </c>
       <c r="D7" t="s">
+        <v>23</v>
+      </c>
+      <c r="E7" t="s">
+        <v>65</v>
+      </c>
+      <c r="H7" t="s">
         <v>24</v>
       </c>
-      <c r="E7" t="s">
-        <v>71</v>
-      </c>
-      <c r="H7" t="s">
+      <c r="J7" s="3" t="s">
         <v>25</v>
-      </c>
-      <c r="J7" s="3" t="s">
-        <v>26</v>
       </c>
       <c r="K7" s="1"/>
     </row>
@@ -930,10 +939,10 @@
         <v>10</v>
       </c>
       <c r="E8" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="H8" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="K8" s="1"/>
     </row>
@@ -948,13 +957,13 @@
         <v>0.70833333333333337</v>
       </c>
       <c r="D9" t="s">
-        <v>28</v>
+        <v>10</v>
       </c>
       <c r="E9" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="H9" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="K9" s="1"/>
     </row>
@@ -969,16 +978,16 @@
         <v>0.91666666666666663</v>
       </c>
       <c r="D10" t="s">
+        <v>28</v>
+      </c>
+      <c r="E10" t="s">
+        <v>69</v>
+      </c>
+      <c r="H10" t="s">
+        <v>29</v>
+      </c>
+      <c r="J10" s="3" t="s">
         <v>30</v>
-      </c>
-      <c r="E10" t="s">
-        <v>75</v>
-      </c>
-      <c r="H10" t="s">
-        <v>31</v>
-      </c>
-      <c r="J10" s="3" t="s">
-        <v>32</v>
       </c>
       <c r="K10" s="1"/>
     </row>
@@ -993,28 +1002,31 @@
         <v>0.83333333333333337</v>
       </c>
       <c r="D11" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="E11" t="s">
-        <v>72</v>
+        <v>66</v>
       </c>
       <c r="H11" t="s">
-        <v>34</v>
+        <v>11</v>
       </c>
       <c r="I11" t="s">
-        <v>91</v>
+        <v>85</v>
+      </c>
+      <c r="J11" s="3" t="s">
+        <v>88</v>
       </c>
       <c r="K11" s="1" t="s">
-        <v>87</v>
+        <v>81</v>
       </c>
       <c r="L11" s="3" t="s">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="M11" s="4" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.2">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13" ht="17" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>5</v>
       </c>
@@ -1025,19 +1037,22 @@
         <v>0.875</v>
       </c>
       <c r="D12" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="E12" t="s">
-        <v>72</v>
+        <v>66</v>
       </c>
       <c r="G12" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="H12" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.2">
+        <v>89</v>
+      </c>
+      <c r="J12" s="3" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" ht="17" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>5</v>
       </c>
@@ -1048,19 +1063,22 @@
         <v>0.91666666666666663</v>
       </c>
       <c r="D13" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="E13" t="s">
-        <v>72</v>
+        <v>66</v>
       </c>
       <c r="G13" t="s">
+        <v>86</v>
+      </c>
+      <c r="H13" t="s">
+        <v>16</v>
+      </c>
+      <c r="J13" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="H13" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.2">
+    </row>
+    <row r="14" spans="1:13" ht="17" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>5</v>
       </c>
@@ -1071,19 +1089,22 @@
         <v>0.95833333333333337</v>
       </c>
       <c r="D14" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="E14" t="s">
-        <v>72</v>
+        <v>66</v>
       </c>
       <c r="G14" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="H14" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.2">
+        <v>32</v>
+      </c>
+      <c r="J14" s="3" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13" ht="17" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>5</v>
       </c>
@@ -1094,16 +1115,19 @@
         <v>0</v>
       </c>
       <c r="D15" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="E15" t="s">
-        <v>72</v>
+        <v>66</v>
       </c>
       <c r="G15" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="H15" t="s">
-        <v>37</v>
+        <v>93</v>
+      </c>
+      <c r="J15" s="3" t="s">
+        <v>94</v>
       </c>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.2">
@@ -1120,13 +1144,13 @@
         <v>14</v>
       </c>
       <c r="E16" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="G16" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="H16" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.2">
@@ -1143,13 +1167,13 @@
         <v>14</v>
       </c>
       <c r="E17" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="G17" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="H17" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.2">
@@ -1166,13 +1190,13 @@
         <v>14</v>
       </c>
       <c r="E18" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="G18" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="H18" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.2">
@@ -1189,10 +1213,10 @@
         <v>14</v>
       </c>
       <c r="E19" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="H19" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.2">
@@ -1209,13 +1233,13 @@
         <v>14</v>
       </c>
       <c r="E20" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="G20" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="H20" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.2">
@@ -1232,13 +1256,13 @@
         <v>14</v>
       </c>
       <c r="E21" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="G21" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="H21" t="s">
-        <v>44</v>
+        <v>38</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.2">
@@ -1255,13 +1279,13 @@
         <v>14</v>
       </c>
       <c r="E22" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="G22" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="H22" t="s">
-        <v>45</v>
+        <v>39</v>
       </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.2">
@@ -1278,13 +1302,13 @@
         <v>14</v>
       </c>
       <c r="E23" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="G23" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="H23" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.2">
@@ -1301,13 +1325,13 @@
         <v>14</v>
       </c>
       <c r="E24" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="G24" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="H24" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.2">
@@ -1324,13 +1348,13 @@
         <v>14</v>
       </c>
       <c r="E25" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="G25" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="H25" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.2">
@@ -1347,13 +1371,13 @@
         <v>14</v>
       </c>
       <c r="E26" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="G26" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="H26" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.2">
@@ -1367,13 +1391,13 @@
         <v>0.8125</v>
       </c>
       <c r="D27" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="E27" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="H27" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.2">
@@ -1387,16 +1411,16 @@
         <v>0.83333333333333337</v>
       </c>
       <c r="D28" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="E28" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="G28" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="H28" t="s">
-        <v>52</v>
+        <v>46</v>
       </c>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.2">
@@ -1410,16 +1434,16 @@
         <v>0.875</v>
       </c>
       <c r="D29" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="E29" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="G29" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="H29" t="s">
-        <v>53</v>
+        <v>47</v>
       </c>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.2">
@@ -1433,16 +1457,16 @@
         <v>0.89583333333333304</v>
       </c>
       <c r="D30" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="E30" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="G30" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="H30" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.2">
@@ -1456,16 +1480,16 @@
         <v>0.91666666666666696</v>
       </c>
       <c r="D31" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="E31" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="G31" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="H31" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.2">
@@ -1479,16 +1503,16 @@
         <v>0.9375</v>
       </c>
       <c r="D32" t="s">
+        <v>44</v>
+      </c>
+      <c r="E32" t="s">
+        <v>67</v>
+      </c>
+      <c r="G32" t="s">
+        <v>86</v>
+      </c>
+      <c r="H32" t="s">
         <v>50</v>
-      </c>
-      <c r="E32" t="s">
-        <v>73</v>
-      </c>
-      <c r="G32" t="s">
-        <v>92</v>
-      </c>
-      <c r="H32" t="s">
-        <v>56</v>
       </c>
     </row>
     <row r="33" spans="1:13" x14ac:dyDescent="0.2">
@@ -1502,16 +1526,16 @@
         <v>0.95833333333333404</v>
       </c>
       <c r="D33" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="E33" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="G33" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="H33" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
     </row>
     <row r="34" spans="1:13" x14ac:dyDescent="0.2">
@@ -1525,16 +1549,16 @@
         <v>0.97916666666666696</v>
       </c>
       <c r="D34" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="E34" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="G34" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="H34" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
     </row>
     <row r="35" spans="1:13" x14ac:dyDescent="0.2">
@@ -1548,16 +1572,16 @@
         <v>1</v>
       </c>
       <c r="D35" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="E35" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="G35" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="H35" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
     </row>
     <row r="36" spans="1:13" x14ac:dyDescent="0.2">
@@ -1571,16 +1595,16 @@
         <v>1.0208333333333299</v>
       </c>
       <c r="D36" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="E36" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="G36" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="H36" t="s">
-        <v>60</v>
+        <v>54</v>
       </c>
     </row>
     <row r="37" spans="1:13" x14ac:dyDescent="0.2">
@@ -1594,16 +1618,16 @@
         <v>1.0416666666666701</v>
       </c>
       <c r="D37" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="E37" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="G37" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="H37" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
     </row>
     <row r="38" spans="1:13" ht="51" x14ac:dyDescent="0.2">
@@ -1617,28 +1641,28 @@
         <v>0.58333333333333337</v>
       </c>
       <c r="D38" t="s">
-        <v>62</v>
+        <v>56</v>
       </c>
       <c r="E38" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="F38" t="s">
-        <v>84</v>
+        <v>78</v>
       </c>
       <c r="G38" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="H38" t="s">
-        <v>63</v>
+        <v>57</v>
       </c>
       <c r="J38" s="3" t="s">
-        <v>64</v>
+        <v>58</v>
       </c>
       <c r="L38" s="3" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="M38" t="s">
-        <v>79</v>
+        <v>73</v>
       </c>
     </row>
     <row r="39" spans="1:13" ht="51" x14ac:dyDescent="0.2">
@@ -1652,28 +1676,28 @@
         <v>0.73958333333333337</v>
       </c>
       <c r="D39" t="s">
-        <v>65</v>
+        <v>59</v>
       </c>
       <c r="E39" t="s">
+        <v>68</v>
+      </c>
+      <c r="F39" t="s">
+        <v>78</v>
+      </c>
+      <c r="G39" t="s">
+        <v>86</v>
+      </c>
+      <c r="H39" t="s">
+        <v>60</v>
+      </c>
+      <c r="J39" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="L39" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="M39" t="s">
         <v>74</v>
-      </c>
-      <c r="F39" t="s">
-        <v>84</v>
-      </c>
-      <c r="G39" t="s">
-        <v>92</v>
-      </c>
-      <c r="H39" t="s">
-        <v>66</v>
-      </c>
-      <c r="J39" s="3" t="s">
-        <v>67</v>
-      </c>
-      <c r="L39" s="3" t="s">
-        <v>77</v>
-      </c>
-      <c r="M39" t="s">
-        <v>80</v>
       </c>
     </row>
     <row r="40" spans="1:13" ht="68" x14ac:dyDescent="0.2">
@@ -1690,28 +1714,28 @@
         <v>15</v>
       </c>
       <c r="E40" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="F40" t="s">
-        <v>84</v>
+        <v>78</v>
       </c>
       <c r="G40" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="H40" t="s">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="J40" s="3" t="s">
-        <v>69</v>
+        <v>63</v>
       </c>
       <c r="K40" s="1" t="s">
-        <v>88</v>
+        <v>82</v>
       </c>
       <c r="L40" s="3" t="s">
-        <v>78</v>
+        <v>72</v>
       </c>
       <c r="M40" t="s">
-        <v>81</v>
+        <v>75</v>
       </c>
     </row>
   </sheetData>

</xml_diff>